<commit_message>
Add sample data to costing template
</commit_message>
<xml_diff>
--- a/cleopatra-delights-costing-template.xlsx
+++ b/cleopatra-delights-costing-template.xlsx
@@ -469,6 +469,25 @@
       </c>
     </row>
     <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>FLOUR_AP</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>All-purpose flour</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>1000</v>
+      </c>
+      <c r="D2" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="E2" t="n">
+        <v>364</v>
+      </c>
       <c r="F2">
         <f>IFERROR(D2/C2,0)</f>
         <v/>
@@ -479,6 +498,25 @@
       </c>
     </row>
     <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>SUGAR_WHT</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>White sugar</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>1000</v>
+      </c>
+      <c r="D3" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="E3" t="n">
+        <v>400</v>
+      </c>
       <c r="F3">
         <f>IFERROR(D3/C3,0)</f>
         <v/>
@@ -489,6 +527,25 @@
       </c>
     </row>
     <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>BUTTER_UNS</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Unsalted butter</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>250</v>
+      </c>
+      <c r="D4" t="n">
+        <v>3</v>
+      </c>
+      <c r="E4" t="n">
+        <v>717</v>
+      </c>
       <c r="F4">
         <f>IFERROR(D4/C4,0)</f>
         <v/>
@@ -499,6 +556,25 @@
       </c>
     </row>
     <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>CHOC_CHIP</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Chocolate chips</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>1000</v>
+      </c>
+      <c r="D5" t="n">
+        <v>5</v>
+      </c>
+      <c r="E5" t="n">
+        <v>480</v>
+      </c>
       <c r="F5">
         <f>IFERROR(D5/C5,0)</f>
         <v/>
@@ -509,6 +585,25 @@
       </c>
     </row>
     <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>MILK_WHOLE</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Whole milk</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>1000</v>
+      </c>
+      <c r="D6" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="E6" t="n">
+        <v>64</v>
+      </c>
       <c r="F6">
         <f>IFERROR(D6/C6,0)</f>
         <v/>
@@ -5519,6 +5614,19 @@
       </c>
     </row>
     <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>CHOCO_COOKIE</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>FLOUR_AP</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>300</v>
+      </c>
       <c r="D2">
         <f>IFERROR(INDEX(Ingredients!$F$2:$F$500,MATCH(B2,Ingredients!$A$2:$A$500,0)),0)</f>
         <v/>
@@ -5537,6 +5645,19 @@
       </c>
     </row>
     <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>CHOCO_COOKIE</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>SUGAR_WHT</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>150</v>
+      </c>
       <c r="D3">
         <f>IFERROR(INDEX(Ingredients!$F$2:$F$500,MATCH(B3,Ingredients!$A$2:$A$500,0)),0)</f>
         <v/>
@@ -5555,6 +5676,19 @@
       </c>
     </row>
     <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>CHOCO_COOKIE</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>BUTTER_UNS</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>200</v>
+      </c>
       <c r="D4">
         <f>IFERROR(INDEX(Ingredients!$F$2:$F$500,MATCH(B4,Ingredients!$A$2:$A$500,0)),0)</f>
         <v/>
@@ -5573,6 +5707,19 @@
       </c>
     </row>
     <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>CHOCO_COOKIE</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>CHOC_CHIP</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>150</v>
+      </c>
       <c r="D5">
         <f>IFERROR(INDEX(Ingredients!$F$2:$F$500,MATCH(B5,Ingredients!$A$2:$A$500,0)),0)</f>
         <v/>
@@ -5591,6 +5738,19 @@
       </c>
     </row>
     <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>CINN_ROLL</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>FLOUR_AP</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>500</v>
+      </c>
       <c r="D6">
         <f>IFERROR(INDEX(Ingredients!$F$2:$F$500,MATCH(B6,Ingredients!$A$2:$A$500,0)),0)</f>
         <v/>
@@ -5609,6 +5769,19 @@
       </c>
     </row>
     <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>CINN_ROLL</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>SUGAR_WHT</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>80</v>
+      </c>
       <c r="D7">
         <f>IFERROR(INDEX(Ingredients!$F$2:$F$500,MATCH(B7,Ingredients!$A$2:$A$500,0)),0)</f>
         <v/>
@@ -5627,6 +5800,19 @@
       </c>
     </row>
     <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>CINN_ROLL</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>BUTTER_UNS</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>120</v>
+      </c>
       <c r="D8">
         <f>IFERROR(INDEX(Ingredients!$F$2:$F$500,MATCH(B8,Ingredients!$A$2:$A$500,0)),0)</f>
         <v/>
@@ -5645,6 +5831,19 @@
       </c>
     </row>
     <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>CINN_ROLL</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>MILK_WHOLE</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>200</v>
+      </c>
       <c r="D9">
         <f>IFERROR(INDEX(Ingredients!$F$2:$F$500,MATCH(B9,Ingredients!$A$2:$A$500,0)),0)</f>
         <v/>
@@ -14585,6 +14784,24 @@
       </c>
     </row>
     <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>CHOCO_COOKIE</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Chocolate Chip Cookies</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>24</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>cookie</t>
+        </is>
+      </c>
       <c r="E2">
         <f>IFERROR(SUMIF(Recipe_Ingredients!$A$2:$A$500,A2,Recipe_Ingredients!$E$2:$E$500),0)</f>
         <v/>
@@ -14601,6 +14818,9 @@
         <f>IFERROR(G2/C2,0)</f>
         <v/>
       </c>
+      <c r="I2" t="n">
+        <v>1.5</v>
+      </c>
       <c r="J2">
         <f>ROUND(F2*3,2)</f>
         <v/>
@@ -14611,6 +14831,24 @@
       </c>
     </row>
     <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>CINN_ROLL</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Cinnamon Rolls</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>12</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>roll</t>
+        </is>
+      </c>
       <c r="E3">
         <f>IFERROR(SUMIF(Recipe_Ingredients!$A$2:$A$500,A3,Recipe_Ingredients!$E$2:$E$500),0)</f>
         <v/>
@@ -14626,6 +14864,9 @@
       <c r="H3">
         <f>IFERROR(G3/C3,0)</f>
         <v/>
+      </c>
+      <c r="I3" t="n">
+        <v>2.5</v>
       </c>
       <c r="J3">
         <f>ROUND(F3*3,2)</f>
@@ -27582,9 +27823,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-    </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -27676,9 +27915,7 @@
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="inlineStr"/>
-    </row>
+    <row r="16"/>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>

</xml_diff>